<commit_message>
Update bundled reimbursement template
</commit_message>
<xml_diff>
--- a/organize-reimbursement/assets/费用报销单模板.xlsx
+++ b/organize-reimbursement/assets/费用报销单模板.xlsx
@@ -9,9 +9,6 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="类别">#REF!</definedName>
   </definedNames>
@@ -71,7 +68,7 @@
     <t>金额</t>
   </si>
   <si>
-    <t>是否增值税发票</t>
+    <t>是否有发票</t>
   </si>
   <si>
     <t>备注</t>
@@ -1316,19 +1313,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="报销单"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
   <a:themeElements>

</xml_diff>